<commit_message>
Updated to use single quotes for sql statements
</commit_message>
<xml_diff>
--- a/reference/Navy Sources and Data Processing/Designators and Billet Codes/EXCEL Spreadsheet for Designators.xlsx
+++ b/reference/Navy Sources and Data Processing/Designators and Billet Codes/EXCEL Spreadsheet for Designators.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael/Development/StudioProjects/NavyDecoder-OpenSource/reference/Navy Sources and Data Processing/Designators and Billet Codes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1147CB9E-BBF1-9845-8DF9-238E9A2C4594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{616F7353-DD6F-124C-9765-ABEB2B758336}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38400" yWindow="600" windowWidth="37860" windowHeight="21000" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4584,8 +4584,10 @@
         <v xml:space="preserve">						{"1000", "Billet which may be filled by any appropriately skilled and experienced Unrestricted Line Officer or Special Duty Officer"},</v>
       </c>
       <c r="E2" s="21" t="str">
-        <f>+_xlfn.CONCAT("insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values (""",B2,""",""",TRIM(C2),""",""NAVPERS 15839I VOL I (JAN 2026)"");")</f>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1000","Billet which may be filled by any appropriately skilled and experienced Unrestricted Line Officer or Special Duty Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <f>"insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('"
+ &amp; SUBSTITUTE(B2,"'","''") &amp; "','"
+ &amp; SUBSTITUTE(TRIM(C2),"'","''") &amp; "','NAVPERS 15839I VOL I (JAN 2026)');"</f>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1000','Billet which may be filled by any appropriately skilled and experienced Unrestricted Line Officer or Special Duty Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -4604,8 +4606,10 @@
         <v xml:space="preserve">						{"1020", "Billet which may be filled by any appropriately skilled and experienced Special Duty Officer (IP) or Unrestricted Line Officer"},</v>
       </c>
       <c r="E3" s="21" t="str">
-        <f t="shared" ref="E3:E66" si="2">+_xlfn.CONCAT("insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values (""",B3,""",""",TRIM(C3),""",""NAVPERS 15839I VOL I (JAN 2026)"");")</f>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1020","Billet which may be filled by any appropriately skilled and experienced Special Duty Officer (IP) or Unrestricted Line Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <f t="shared" ref="E3:E66" si="2">"insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('"
+ &amp; SUBSTITUTE(B3,"'","''") &amp; "','"
+ &amp; SUBSTITUTE(TRIM(C3),"'","''") &amp; "','NAVPERS 15839I VOL I (JAN 2026)');"</f>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1020','Billet which may be filled by any appropriately skilled and experienced Special Duty Officer (IP) or Unrestricted Line Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -4625,7 +4629,7 @@
       </c>
       <c r="E4" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1050","Unrestricted Line Officer billet requiring an officer qualified in any one of the warfare specialties (LT and above)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1050','Unrestricted Line Officer billet requiring an officer qualified in any one of the warfare specialties (LT and above)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -4645,7 +4649,7 @@
       </c>
       <c r="E5" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1100","Unrestricted Line Officer billet requiring Fleet Support specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1100','Unrestricted Line Officer billet requiring Fleet Support specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -4665,7 +4669,7 @@
       </c>
       <c r="E6" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1110","Unrestricted Line Officer billet requiring Surface Warfare qualification or afloat billets leading to such qualification","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1110','Unrestricted Line Officer billet requiring Surface Warfare qualification or afloat billets leading to such qualification','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -4685,7 +4689,7 @@
       </c>
       <c r="E7" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1120","Unrestricted Line Officer billet requiring Submarine Warfare qualification or afloat billets leading to such qualification","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1120','Unrestricted Line Officer billet requiring Submarine Warfare qualification or afloat billets leading to such qualification','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -4705,7 +4709,7 @@
       </c>
       <c r="E8" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1130","Unrestricted Line Officer billet requiring Special Warfare (SEAL) qualification","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1130','Unrestricted Line Officer billet requiring Special Warfare (SEAL) qualification','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -4725,7 +4729,7 @@
       </c>
       <c r="E9" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1140","Unrestricted Line Officer billet requiring Explosive Ordnance Disposal (EOD) Warfare Qualification","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1140','Unrestricted Line Officer billet requiring Explosive Ordnance Disposal (EOD) Warfare Qualification','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -4745,7 +4749,7 @@
       </c>
       <c r="E10" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1160","Unrestricted Line Officer billet for an officer in training for Surface Warfare qualification","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1160','Unrestricted Line Officer billet for an officer in training for Surface Warfare qualification','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -4765,7 +4769,7 @@
       </c>
       <c r="E11" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1170","Unrestricted Line Officer billet for an officer in training for Submarine Warfare qualification","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1170','Unrestricted Line Officer billet for an officer in training for Submarine Warfare qualification','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -4785,7 +4789,7 @@
       </c>
       <c r="E12" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1180","Unrestricted Line Officer billet for a student in training for Special Warfare qualification","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1180','Unrestricted Line Officer billet for a student in training for Special Warfare qualification','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -4805,10 +4809,10 @@
       </c>
       <c r="E13" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1190","Unrestricted Line Officer billet for an officer in training for Explosive Ordnance Disposal (EOD) qualification","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1190','Unrestricted Line Officer billet for an officer in training for Explosive Ordnance Disposal (EOD) qualification','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A14" s="25">
         <v>1200</v>
       </c>
@@ -4825,10 +4829,10 @@
       </c>
       <c r="E14" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1200","Special Duty Officer - Restricted Line Officer Billet requiring Human Resources specialty - Plan, program, and execute life-cycle management of our Navy's most important resource - people.","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1200','Special Duty Officer - Restricted Line Officer Billet requiring Human Resources specialty - Plan, program, and execute life-cycle management of our Navy''s most important resource - people.','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A15" s="25">
         <v>1210</v>
       </c>
@@ -4845,7 +4849,7 @@
       </c>
       <c r="E15" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1210","Restricted Line Officer Billet (Nuclear Power School Instructor) regulated by Program Authorization 100B attached to Nuclear Power School, Charleston, SC.","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1210','Restricted Line Officer Billet (Nuclear Power School Instructor) regulated by Program Authorization 100B attached to Nuclear Power School, Charleston, SC.','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -4865,7 +4869,7 @@
       </c>
       <c r="E16" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1230","Restricted Line Officer Billet (Permanent Military Professor) regulated by OPNAVINST 1520.40","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1230','Restricted Line Officer Billet (Permanent Military Professor) regulated by OPNAVINST 1520.40','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -4885,10 +4889,10 @@
       </c>
       <c r="E17" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1280","Special Duty Officer-Restricted Line Officer Billet Requiring Recruiting Specialty of a permanent Recruiter (LT and LCDR)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1280','Special Duty Officer-Restricted Line Officer Billet Requiring Recruiting Specialty of a permanent Recruiter (LT and LCDR)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A18" s="25" t="s">
         <v>59</v>
       </c>
@@ -4905,7 +4909,7 @@
       </c>
       <c r="E18" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1300","Unrestricted Line Officer billet, Code 0 - Other Than Operational Flying, requiring Air Warfare specialty of, or previous designation as, a pilot or NFO (LT and above)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1300','Unrestricted Line Officer billet, Code 0 - Other Than Operational Flying, requiring Air Warfare specialty of, or previous designation as, a pilot or NFO (LT and above)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -4925,7 +4929,7 @@
       </c>
       <c r="E19" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1301","Unrestricted Line Officer billet, Code 1 - Operational Flying, requiring Air Warfare specialty of a pilot or NFO (LT and above)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1301','Unrestricted Line Officer billet, Code 1 - Operational Flying, requiring Air Warfare specialty of a pilot or NFO (LT and above)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -4945,7 +4949,7 @@
       </c>
       <c r="E20" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1302","Unrestricted Line Officer billet, Code 2 - Operational Flying, requiring Air Warfare specialty of a pilot or NFO","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1302','Unrestricted Line Officer billet, Code 2 - Operational Flying, requiring Air Warfare specialty of a pilot or NFO','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -4965,7 +4969,7 @@
       </c>
       <c r="E21" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1310","Unrestricted Line Officer billet, Code 0 - Other Than Operational Flying, requiring Aviation Warfare specialty of a pilot","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1310','Unrestricted Line Officer billet, Code 0 - Other Than Operational Flying, requiring Aviation Warfare specialty of a pilot','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -4985,7 +4989,7 @@
       </c>
       <c r="E22" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1311","Unrestricted Line Officer billet, Code 1 - Operational Flying, requiring Aviation Warfare specialty of a pilot","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1311','Unrestricted Line Officer billet, Code 1 - Operational Flying, requiring Aviation Warfare specialty of a pilot','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5005,10 +5009,10 @@
       </c>
       <c r="E23" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1312","Unrestricted Line Officer billet, Code 2 - Operational Flying, requiring Aviation Warfare specialty of a pilot","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1312','Unrestricted Line Officer billet, Code 2 - Operational Flying, requiring Aviation Warfare specialty of a pilot','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A24" s="25" t="s">
         <v>76</v>
       </c>
@@ -5025,7 +5029,7 @@
       </c>
       <c r="E24" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1320","Unrestricted Line Officer billet, Code 0 - Other Than Operational Flying, requiring Aviation Warfare specialty of a Naval Flight Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1320','Unrestricted Line Officer billet, Code 0 - Other Than Operational Flying, requiring Aviation Warfare specialty of a Naval Flight Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5045,7 +5049,7 @@
       </c>
       <c r="E25" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1321","Unrestricted Line Officer billet, Code 1 - Operational Flying, requiring Aviation Warfare specialty of a Naval Flight Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1321','Unrestricted Line Officer billet, Code 1 - Operational Flying, requiring Aviation Warfare specialty of a Naval Flight Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5065,7 +5069,7 @@
       </c>
       <c r="E26" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1322","Unrestricted Line Officer billet, Code 2 - Operational Flying, requiring Aviation Warfare specialty of a Naval Flight Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1322','Unrestricted Line Officer billet, Code 2 - Operational Flying, requiring Aviation Warfare specialty of a Naval Flight Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5085,7 +5089,7 @@
       </c>
       <c r="E27" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1372","Unrestricted Line Officer billet, Code 2 - Operational Flying, for a student in training for Aviation Warfare (NFO) qualification","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1372','Unrestricted Line Officer billet, Code 2 - Operational Flying, for a student in training for Aviation Warfare (NFO) qualification','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5105,10 +5109,10 @@
       </c>
       <c r="E28" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1392","Unrestricted Line Officer billet, Code 2 - Operational Flying, for a student in training for Aviation Warfare (pilot) qualification","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="70" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1392','Unrestricted Line Officer billet, Code 2 - Operational Flying, for a student in training for Aviation Warfare (pilot) qualification','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A29" s="25">
         <v>1440</v>
       </c>
@@ -5125,7 +5129,7 @@
       </c>
       <c r="E29" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1440","Engineering Duty Officer billet requiring specialists in Ship Engineering, including Ship and Ship Systems Engineering, Electronic Systems Engineering, Combat/Weapons Systems Engineering, and Ordnance Systems Engineering.","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1440','Engineering Duty Officer billet requiring specialists in Ship Engineering, including Ship and Ship Systems Engineering, Electronic Systems Engineering, Combat/Weapons Systems Engineering, and Ordnance Systems Engineering.','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5145,10 +5149,10 @@
       </c>
       <c r="E30" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1460","Engineering Duty Officer billet for an officer actively pursuing a prescribed program leading to designation as 144X","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1460','Engineering Duty Officer billet for an officer actively pursuing a prescribed program leading to designation as 144X','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A31" s="25">
         <v>1500</v>
       </c>
@@ -5165,7 +5169,7 @@
       </c>
       <c r="E31" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1500","Aerospace Engineering Duty Officer billet requiring Aerospace Engineering (AED) or Aerospace maintenance (AMD) specialties (CAPT and above)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1500','Aerospace Engineering Duty Officer billet requiring Aerospace Engineering (AED) or Aerospace maintenance (AMD) specialties (CAPT and above)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5185,10 +5189,10 @@
       </c>
       <c r="E32" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1510","Aerospace Engineering Duty Officer billet requiring Aerospace Engineering (AED) specialty.","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1510','Aerospace Engineering Duty Officer billet requiring Aerospace Engineering (AED) specialty.','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A33" s="25" t="s">
         <v>111</v>
       </c>
@@ -5205,10 +5209,10 @@
       </c>
       <c r="E33" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1511","Aerospace Engineering Duty Officer billet, Code 1 - Operational Flying, requiring the specialty of an Aerospace Engineering Duty (AED) officer who is a designated Pilot or Naval Flight Officer.","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1511','Aerospace Engineering Duty Officer billet, Code 1 - Operational Flying, requiring the specialty of an Aerospace Engineering Duty (AED) officer who is a designated Pilot or Naval Flight Officer.','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A34" s="25" t="s">
         <v>112</v>
       </c>
@@ -5225,10 +5229,10 @@
       </c>
       <c r="E34" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1512","Aerospace Engineering Duty Officer billet, Code 2 - Operational Flying, requiring the specialty of an Aerospace Engineering Duty (AED) Officer who is a designated Pilot or Naval Flight Officer.","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1512','Aerospace Engineering Duty Officer billet, Code 2 - Operational Flying, requiring the specialty of an Aerospace Engineering Duty (AED) Officer who is a designated Pilot or Naval Flight Officer.','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A35" s="25" t="s">
         <v>113</v>
       </c>
@@ -5245,7 +5249,7 @@
       </c>
       <c r="E35" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1540","Aviation Duty Officer billet, Code 0 - Other Than Operational Flying, requiring Aviation Warfare specialty of a pilot (LT thru CAPT)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1540','Aviation Duty Officer billet, Code 0 - Other Than Operational Flying, requiring Aviation Warfare specialty of a pilot (LT thru CAPT)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5265,7 +5269,7 @@
       </c>
       <c r="E36" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1541","Aviation Duty Officer billet, Code 1 - Operational Flying, requiring Aviation Warfare specialty of a pilot (LT thru CAPT)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1541','Aviation Duty Officer billet, Code 1 - Operational Flying, requiring Aviation Warfare specialty of a pilot (LT thru CAPT)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5285,7 +5289,7 @@
       </c>
       <c r="E37" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1542","Aviation Duty Officer billet, Code 2 - Operational Flying, requiring Aviation Warfare specialty of a pilot (LT thru CAPT)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1542','Aviation Duty Officer billet, Code 2 - Operational Flying, requiring Aviation Warfare specialty of a pilot (LT thru CAPT)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5305,7 +5309,7 @@
       </c>
       <c r="E38" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1650","Special Duty Officer billet requiring Public Affairs specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1650','Special Duty Officer billet requiring Public Affairs specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5325,7 +5329,7 @@
       </c>
       <c r="E39" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1660","Special Duty Officer billet requiring a Strategic Sealift Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1660','Special Duty Officer billet requiring a Strategic Sealift Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5345,10 +5349,10 @@
       </c>
       <c r="E40" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1710","Special Duty Officer billet requiring a qualified Foreign Area Officer or a Foreign Area Officer Under Instruction","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1710','Special Duty Officer billet requiring a qualified Foreign Area Officer or a Foreign Area Officer Under Instruction','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A41" s="25">
         <v>1712</v>
       </c>
@@ -5365,7 +5369,7 @@
       </c>
       <c r="E41" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1712","Special Duty Officer billet requiring a Foreign Area Officer Code 2 – Operational Flying Involved, a qualified Foreign Area Officer or a Foreign Area Officer Under Instruction","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1712','Special Duty Officer billet requiring a Foreign Area Officer Code 2 – Operational Flying Involved, a qualified Foreign Area Officer or a Foreign Area Officer Under Instruction','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5385,10 +5389,10 @@
       </c>
       <c r="E42" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1800","Information Warfare Line Officer - Oceanography","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1800','Information Warfare Line Officer - Oceanography','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A43" s="25" t="s">
         <v>145</v>
       </c>
@@ -5405,7 +5409,7 @@
       </c>
       <c r="E43" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1802","Information Warfare Line Officer billet Code 2 - Operational Flying, requiring Meteorology specialty of a Geophysicist who is a designated Pilot or Naval Flight Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1802','Information Warfare Line Officer billet Code 2 - Operational Flying, requiring Meteorology specialty of a Geophysicist who is a designated Pilot or Naval Flight Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5425,7 +5429,7 @@
       </c>
       <c r="E44" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1810","Information Warfare Line Officer – Cryptologic Warfare Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1810','Information Warfare Line Officer – Cryptologic Warfare Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5445,7 +5449,7 @@
       </c>
       <c r="E45" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1820","Information Warfare Line Officer – Information Professional Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1820','Information Warfare Line Officer – Information Professional Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5465,7 +5469,7 @@
       </c>
       <c r="E46" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1830","Information Warfare Line Officer – Intelligence Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1830','Information Warfare Line Officer – Intelligence Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5485,7 +5489,7 @@
       </c>
       <c r="E47" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1840","Information Warfare Line Officer – Cyber Warfare Engineer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1840','Information Warfare Line Officer – Cyber Warfare Engineer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5505,7 +5509,7 @@
       </c>
       <c r="E48" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1850","Billets which may be filled by any appropriately skilled and experienced IWC Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1850','Billets which may be filled by any appropriately skilled and experienced IWC Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5525,10 +5529,10 @@
       </c>
       <c r="E49" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1860","Information Warfare Line Officer – IWC Flag Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1860','Information Warfare Line Officer – IWC Flag Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A50" s="25">
         <v>1870</v>
       </c>
@@ -5545,7 +5549,7 @@
       </c>
       <c r="E50" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1870","Information Warfare Line Officer – Maritime Space Officer / Warfare –qualified URL/RL officers at O3, O4, O5 and O6 level / Reserve Grades URL/RL O2 to O6","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1870','Information Warfare Line Officer – Maritime Space Officer / Warfare –qualified URL/RL officers at O3, O4, O5 and O6 level / Reserve Grades URL/RL O2 to O6','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5565,7 +5569,7 @@
       </c>
       <c r="E51" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1880","Information Warfare Line Officer -Maritime Cyber Warfare Officer (O1 to O6)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1880','Information Warfare Line Officer -Maritime Cyber Warfare Officer (O1 to O6)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5585,7 +5589,7 @@
       </c>
       <c r="E52" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1900","Unrestricted Line Officer student billet for a prospective Nurse Corps officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1900','Unrestricted Line Officer student billet for a prospective Nurse Corps officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5605,7 +5609,7 @@
       </c>
       <c r="E53" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1910","Unrestricted Line Officer student billet for a prospective Medical Corps officer (Senior Medical Student Program)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1910','Unrestricted Line Officer student billet for a prospective Medical Corps officer (Senior Medical Student Program)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5625,7 +5629,7 @@
       </c>
       <c r="E54" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1920","Unrestricted Line Officer student billet for a prospective Dental Corps officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1920','Unrestricted Line Officer student billet for a prospective Dental Corps officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5645,10 +5649,10 @@
       </c>
       <c r="E55" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1930","Unrestricted Line Officer student billet for a prospective Medical Service officer (Optometry)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1930','Unrestricted Line Officer student billet for a prospective Medical Service officer (Optometry)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A56" s="25">
         <v>1950</v>
       </c>
@@ -5665,7 +5669,7 @@
       </c>
       <c r="E56" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1950","Unrestricted Line Officer student billet for a prospective Judge Advocate General’s Corps Officer Law Education Program (LEP)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1950','Unrestricted Line Officer student billet for a prospective Judge Advocate General’s Corps Officer Law Education Program (LEP)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5685,10 +5689,10 @@
       </c>
       <c r="E57" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("1960","Unrestricted Line Officer student billet for a prospective Medical Corps officer (Medical /Osteopathic Scholarship Program)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('1960','Unrestricted Line Officer student billet for a prospective Medical Corps officer (Medical /Osteopathic Scholarship Program)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A58" s="25">
         <v>2000</v>
       </c>
@@ -5705,7 +5709,7 @@
       </c>
       <c r="E58" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("2000","Medical Department (Medical Admin) Officer billet which may be filled by an appropriately skilled and experienced individual of one of the Medical Department officer communities (LCDR and above)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('2000','Medical Department (Medical Admin) Officer billet which may be filled by an appropriately skilled and experienced individual of one of the Medical Department officer communities (LCDR and above)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5725,7 +5729,7 @@
       </c>
       <c r="E59" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("2100","Staff Corps Officer billet requiring Medical specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('2100','Staff Corps Officer billet requiring Medical specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5745,7 +5749,7 @@
       </c>
       <c r="E60" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("2102","Staff Corps Officer billet Code 2 - Operational Flying, requiring Medical specialty of a qualified Flight Surgeon","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('2102','Staff Corps Officer billet Code 2 - Operational Flying, requiring Medical specialty of a qualified Flight Surgeon','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5765,10 +5769,10 @@
       </c>
       <c r="E61" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("2200","Staff Corps Officer billet requiring Dental specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('2200','Staff Corps Officer billet requiring Dental specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A62" s="25">
         <v>2300</v>
       </c>
@@ -5785,10 +5789,10 @@
       </c>
       <c r="E62" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("2300","Staff Corps Officer billet requiring Medical Service (Health Care Administration, Medical Allied Science, Optometry, Pharmacy, or Medical Specialist) specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('2300','Staff Corps Officer billet requiring Medical Service (Health Care Administration, Medical Allied Science, Optometry, Pharmacy, or Medical Specialist) specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A63" s="25" t="s">
         <v>200</v>
       </c>
@@ -5805,7 +5809,7 @@
       </c>
       <c r="E63" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("2302","Staff Corps Officer billet, Code 2 - Operational Flying, requiring specialty of a qualified Aviation Physiologist, Aviation Experimental Psychologist, or Flight Physician Assistant","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('2302','Staff Corps Officer billet, Code 2 - Operational Flying, requiring specialty of a qualified Aviation Physiologist, Aviation Experimental Psychologist, or Flight Physician Assistant','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5825,7 +5829,7 @@
       </c>
       <c r="E64" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("2500","Staff Corps Officer billet requiring Law specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('2500','Staff Corps Officer billet requiring Law specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5845,7 +5849,7 @@
       </c>
       <c r="E65" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("2900","Staff Corps Officer billet requiring Nursing specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('2900','Staff Corps Officer billet requiring Nursing specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5865,7 +5869,7 @@
       </c>
       <c r="E66" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("3100","Staff Corps Officer billet requiring Supply specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('3100','Staff Corps Officer billet requiring Supply specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5884,8 +5888,10 @@
         <v xml:space="preserve">						{"4100", "Staff Corps Officer billet requiring Chaplain specialty"},</v>
       </c>
       <c r="E67" s="21" t="str">
-        <f t="shared" ref="E67:E120" si="5">+_xlfn.CONCAT("insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values (""",B67,""",""",TRIM(C67),""",""NAVPERS 15839I VOL I (JAN 2026)"");")</f>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("4100","Staff Corps Officer billet requiring Chaplain specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <f t="shared" ref="E67:E120" si="5">"insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('"
+ &amp; SUBSTITUTE(B67,"'","''") &amp; "','"
+ &amp; SUBSTITUTE(TRIM(C67),"'","''") &amp; "','NAVPERS 15839I VOL I (JAN 2026)');"</f>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('4100','Staff Corps Officer billet requiring Chaplain specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5905,7 +5911,7 @@
       </c>
       <c r="E68" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("5100","Staff Corps Officer billet requiring Civil Engineering specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('5100','Staff Corps Officer billet requiring Civil Engineering specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5925,7 +5931,7 @@
       </c>
       <c r="E69" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6000","Billet which may be filled by any appropriately skilled and experienced Limited Duty Officer Line (CDR and above)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6000','Billet which may be filled by any appropriately skilled and experienced Limited Duty Officer Line (CDR and above)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5945,7 +5951,7 @@
       </c>
       <c r="E70" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6110","Limited Duty Officer (Line) billet requiring management in Deck specialty (Surface)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6110','Limited Duty Officer (Line) billet requiring management in Deck specialty (Surface)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5965,7 +5971,7 @@
       </c>
       <c r="E71" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6120","Limited Duty Officer (Line) billet requiring management in Operations specialty (Surface)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6120','Limited Duty Officer (Line) billet requiring management in Operations specialty (Surface)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -5985,7 +5991,7 @@
       </c>
       <c r="E72" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6130","Limited Duty Officer (Line) billet requiring management in Engineering/Repair specialty (Surface)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6130','Limited Duty Officer (Line) billet requiring management in Engineering/Repair specialty (Surface)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6005,7 +6011,7 @@
       </c>
       <c r="E73" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6180","Limited Duty Officer (Line) billet requiring management in Electronics specialty (Surface)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6180','Limited Duty Officer (Line) billet requiring management in Electronics specialty (Surface)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6025,7 +6031,7 @@
       </c>
       <c r="E74" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6200","Limited Duty Officer (Line) billet requiring management in Nuclear Power specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6200','Limited Duty Officer (Line) billet requiring management in Nuclear Power specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6045,7 +6051,7 @@
       </c>
       <c r="E75" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6230","Limited Duty Officer (Line) billet requiring management in Engineering/Repair specialty (Submarine)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6230','Limited Duty Officer (Line) billet requiring management in Engineering/Repair specialty (Submarine)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6065,7 +6071,7 @@
       </c>
       <c r="E76" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6260","Limited Duty Officer (Line) billet requiring management in Ordnance specialty (Submarine)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6260','Limited Duty Officer (Line) billet requiring management in Ordnance specialty (Submarine)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6085,7 +6091,7 @@
       </c>
       <c r="E77" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6280","Limited Duty Officer (Line) billet requiring management in Electronics specialty (Submarine)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6280','Limited Duty Officer (Line) billet requiring management in Electronics specialty (Submarine)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6105,7 +6111,7 @@
       </c>
       <c r="E78" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6290","Limited Duty Officer (Line) billet requiring management in Communications specialty (Submarine)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6290','Limited Duty Officer (Line) billet requiring management in Communications specialty (Submarine)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6125,7 +6131,7 @@
       </c>
       <c r="E79" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6310","Limited Duty Officer (Line) billet requiring management in Aviation Deck specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6310','Limited Duty Officer (Line) billet requiring management in Aviation Deck specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6145,10 +6151,10 @@
       </c>
       <c r="E80" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6320","Limited Duty Officer (Line) billet requiring management in Aviation Operations specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6320','Limited Duty Officer (Line) billet requiring management in Aviation Operations specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A81" s="25" t="s">
         <v>261</v>
       </c>
@@ -6165,7 +6171,7 @@
       </c>
       <c r="E81" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6321","Limited Duty Officer (Line) billet, Code 1 - Operational Flying, requiring the specialty of an Aviation Operations (ASW) officer who is aeronautically designated","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6321','Limited Duty Officer (Line) billet, Code 1 - Operational Flying, requiring the specialty of an Aviation Operations (ASW) officer who is aeronautically designated','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="82" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6185,7 +6191,7 @@
       </c>
       <c r="E82" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6330","Limited Duty Officer (Line) billet requiring management in Aviation Maintenance specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6330','Limited Duty Officer (Line) billet requiring management in Aviation Maintenance specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="83" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6205,7 +6211,7 @@
       </c>
       <c r="E83" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6360","Limited Duty Officer (Line) billet requiring management in Aviation Ordnance specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6360','Limited Duty Officer (Line) billet requiring management in Aviation Ordnance specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="84" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6225,7 +6231,7 @@
       </c>
       <c r="E84" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6390","Limited Duty Officer (Line) billet requiring management in Air Traffic Control specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6390','Limited Duty Officer (Line) billet requiring management in Air Traffic Control specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="85" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6245,7 +6251,7 @@
       </c>
       <c r="E85" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6410","Limited Duty Officer (Line) billet requiring management in Administration specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6410','Limited Duty Officer (Line) billet requiring management in Administration specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="86" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6265,7 +6271,7 @@
       </c>
       <c r="E86" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6430","Limited Duty Officer (Line) billet requiring Bandmaster specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6430','Limited Duty Officer (Line) billet requiring Bandmaster specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="87" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6285,7 +6291,7 @@
       </c>
       <c r="E87" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6480","Limited Duty Officer (Line) billet requiring management in Explosive Ordnance Disposal specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6480','Limited Duty Officer (Line) billet requiring management in Explosive Ordnance Disposal specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="88" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6305,7 +6311,7 @@
       </c>
       <c r="E88" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6490","Limited Duty Officer (Line) billet requiring management in Security specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6490','Limited Duty Officer (Line) billet requiring management in Security specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="89" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6325,7 +6331,7 @@
       </c>
       <c r="E89" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6510","Staff Corps Limited Duty Officer billet requiring Supply specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6510','Staff Corps Limited Duty Officer billet requiring Supply specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="90" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6345,7 +6351,7 @@
       </c>
       <c r="E90" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6530","Staff Corps Limited Duty Officer billet requiring Civil Engineering specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6530','Staff Corps Limited Duty Officer billet requiring Civil Engineering specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="91" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6365,7 +6371,7 @@
       </c>
       <c r="E91" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6800","Limited Duty Officer (Line) billet requiring management in Meteorology/Oceanography specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6800','Limited Duty Officer (Line) billet requiring management in Meteorology/Oceanography specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="92" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6385,7 +6391,7 @@
       </c>
       <c r="E92" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6810","Limited Duty Officer (Line) billet requiring management in Cryptologic Warfare specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6810','Limited Duty Officer (Line) billet requiring management in Cryptologic Warfare specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="93" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6405,7 +6411,7 @@
       </c>
       <c r="E93" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6820","Limited Duty Officer (Line) billet requiring management in Information Professional","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6820','Limited Duty Officer (Line) billet requiring management in Information Professional','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="94" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6425,7 +6431,7 @@
       </c>
       <c r="E94" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("6830","Limited Duty Officer (Line) billet requiring management in Intelligence specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('6830','Limited Duty Officer (Line) billet requiring management in Intelligence specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="95" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6445,7 +6451,7 @@
       </c>
       <c r="E95" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7110","Warrant Officer (Line) billet requiring supervision in Boatswain specialty (Surface)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7110','Warrant Officer (Line) billet requiring supervision in Boatswain specialty (Surface)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="96" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6465,7 +6471,7 @@
       </c>
       <c r="E96" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7120","Warrant Officer (Line) billet requiring supervision in Operations Technician specialty (Surface)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7120','Warrant Officer (Line) billet requiring supervision in Operations Technician specialty (Surface)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="97" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6485,7 +6491,7 @@
       </c>
       <c r="E97" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7130","Warrant Officer (Line) billet requiring supervision in Engineering specialty (Surface)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7130','Warrant Officer (Line) billet requiring supervision in Engineering specialty (Surface)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="98" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6505,7 +6511,7 @@
       </c>
       <c r="E98" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7150","Warrant Officer (Line) billet requiring supervision in Special Warfare Technician specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7150','Warrant Officer (Line) billet requiring supervision in Special Warfare Technician specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="99" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6525,7 +6531,7 @@
       </c>
       <c r="E99" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7170","Warrant Officer (Line) billet requiring supervision in Naval Special Warfare Combat Crewman","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7170','Warrant Officer (Line) billet requiring supervision in Naval Special Warfare Combat Crewman','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="100" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6545,7 +6551,7 @@
       </c>
       <c r="E100" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7180","Warrant Officer (Line) billet requiring supervision in Electronics Technician specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7180','Warrant Officer (Line) billet requiring supervision in Electronics Technician specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="101" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6565,7 +6571,7 @@
       </c>
       <c r="E101" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7200","Warrant Officer (Line) billet requiring specialty of a Diving Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7200','Warrant Officer (Line) billet requiring specialty of a Diving Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="102" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6585,7 +6591,7 @@
       </c>
       <c r="E102" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7260","Warrant Officer (Line) billet requiring supervision in Ordnance Technician specialty (Submarine)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7260','Warrant Officer (Line) billet requiring supervision in Ordnance Technician specialty (Submarine)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="103" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6605,7 +6611,7 @@
       </c>
       <c r="E103" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7280","Warrant Officer (Line) billet requiring specialty of an Acoustic Technician","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7280','Warrant Officer (Line) billet requiring specialty of an Acoustic Technician','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="104" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6625,7 +6631,7 @@
       </c>
       <c r="E104" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7310","Warrant Officer (Line) billet requiring supervision in Aviation Boatswain specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7310','Warrant Officer (Line) billet requiring supervision in Aviation Boatswain specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="105" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6645,10 +6651,10 @@
       </c>
       <c r="E105" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7320","Warrant Officer (Line) billet requiring supervision in Aviation Operations Technician specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7320','Warrant Officer (Line) billet requiring supervision in Aviation Operations Technician specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A106" s="25" t="s">
         <v>346</v>
       </c>
@@ -6665,7 +6671,7 @@
       </c>
       <c r="E106" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7321","Warrant Officer (Line) billet, Code 1 - Operational Flying, requiring the specialty of an Aviation Operations (ASW) Technician who is aeronautically designated","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7321','Warrant Officer (Line) billet, Code 1 - Operational Flying, requiring the specialty of an Aviation Operations (ASW) Technician who is aeronautically designated','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="107" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6685,7 +6691,7 @@
       </c>
       <c r="E107" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7330","Warrant Officer (Line) billet requiring supervision in Aviation Maintenance Technician specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7330','Warrant Officer (Line) billet requiring supervision in Aviation Maintenance Technician specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="108" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6705,10 +6711,10 @@
       </c>
       <c r="E108" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7360","Warrant Officer (Line) billet requiring supervision in Aviation Ordnance Technician specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7360','Warrant Officer (Line) billet requiring supervision in Aviation Ordnance Technician specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A109" s="25">
         <v>7371</v>
       </c>
@@ -6725,7 +6731,7 @@
       </c>
       <c r="E109" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7371","Warrant Officer (Line) billet, Code 1 – Operational Flying, requiring the specialty of piloting Unmanned Aerial Vehicles who is aeronautically designated.","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7371','Warrant Officer (Line) billet, Code 1 – Operational Flying, requiring the specialty of piloting Unmanned Aerial Vehicles who is aeronautically designated.','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="110" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6745,7 +6751,7 @@
       </c>
       <c r="E110" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7400","Warrant Officer (Line) billet requiring supervision in Nuclear Power Technician specialty.","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7400','Warrant Officer (Line) billet requiring supervision in Nuclear Power Technician specialty.','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="111" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6765,7 +6771,7 @@
       </c>
       <c r="E111" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7410","Warrant Officer (Line) billet requiring supervision in Ship's Clerk specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7410','Warrant Officer (Line) billet requiring supervision in Ship''s Clerk specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="112" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6785,7 +6791,7 @@
       </c>
       <c r="E112" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7490","Warrant Officer (Line) billet requiring supervision in Security Technician specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7490','Warrant Officer (Line) billet requiring supervision in Security Technician specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="113" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6805,7 +6811,7 @@
       </c>
       <c r="E113" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7520","Warrant Officer (Staff Corps) billet requiring supervision in Food Service specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7520','Warrant Officer (Staff Corps) billet requiring supervision in Food Service specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="114" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6825,7 +6831,7 @@
       </c>
       <c r="E114" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7530","Warrant Officer (Staff Corps) billet requiring supervision in Civil Engineering specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7530','Warrant Officer (Staff Corps) billet requiring supervision in Civil Engineering specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="115" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6845,7 +6851,7 @@
       </c>
       <c r="E115" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7560","Warrant Officer (Staff Corps) billet requiring Technical Nurse specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7560','Warrant Officer (Staff Corps) billet requiring Technical Nurse specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="116" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6865,7 +6871,7 @@
       </c>
       <c r="E116" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7800","Warrant Officer (Line) billet requiring supervision Oceanography","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7800','Warrant Officer (Line) billet requiring supervision Oceanography','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="117" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6885,7 +6891,7 @@
       </c>
       <c r="E117" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7810","Warrant Officer (Line) billet requiring supervision in Cryptologic Warfare Technician specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7810','Warrant Officer (Line) billet requiring supervision in Cryptologic Warfare Technician specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="118" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6905,7 +6911,7 @@
       </c>
       <c r="E118" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7820","Warrant Officer (Line) billet requiring supervision in Information Systems Technician specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7820','Warrant Officer (Line) billet requiring supervision in Information Systems Technician specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="119" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6925,7 +6931,7 @@
       </c>
       <c r="E119" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7830","Warrant Officer (Line) billet requiring supervision in Intelligence Technician specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7830','Warrant Officer (Line) billet requiring supervision in Intelligence Technician specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="120" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -6945,7 +6951,7 @@
       </c>
       <c r="E120" s="21" t="str">
         <f t="shared" si="5"/>
-        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ("7840","Warrant Officer (Line) billet requiring supervision in Cyber Warfare specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_billet_codes (suggest_text_1, suggest_text_2, source) values ('7840','Warrant Officer (Line) billet requiring supervision in Cyber Warfare specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
   </sheetData>
@@ -7001,8 +7007,10 @@
         <v xml:space="preserve">						{"110X", "An Unrestricted Line Officer who is not qualified in any warfare specialty or in training for any warfare specialty"},</v>
       </c>
       <c r="E2" s="21" t="str">
-        <f>+_xlfn.CONCAT("insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values (""",B2,""",""",TRIM(C2),""",""NAVPERS 15839I VOL I (JAN 2026)"");")</f>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("110X","An Unrestricted Line Officer who is not qualified in any warfare specialty or in training for any warfare specialty","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <f>"insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('"
+ &amp; SUBSTITUTE(B2, "'", "''") &amp; "','"
+ &amp; SUBSTITUTE(TRIM(C2), "'", "''") &amp; "','NAVPERS 15839I VOL I (JAN 2026)');"</f>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('110X','An Unrestricted Line Officer who is not qualified in any warfare specialty or in training for any warfare specialty','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7021,8 +7029,10 @@
         <v xml:space="preserve">						{"111X", "An Unrestricted Line Officer who is qualified in Surface Warfare"},</v>
       </c>
       <c r="E3" s="21" t="str">
-        <f t="shared" ref="E3:E66" si="2">+_xlfn.CONCAT("insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values (""",B3,""",""",TRIM(C3),""",""NAVPERS 15839I VOL I (JAN 2026)"");")</f>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("111X","An Unrestricted Line Officer who is qualified in Surface Warfare","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <f t="shared" ref="E3:E66" si="2">"insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('"
+ &amp; SUBSTITUTE(B3, "'", "''") &amp; "','"
+ &amp; SUBSTITUTE(TRIM(C3), "'", "''") &amp; "','NAVPERS 15839I VOL I (JAN 2026)');"</f>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('111X','An Unrestricted Line Officer who is qualified in Surface Warfare','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7042,7 +7052,7 @@
       </c>
       <c r="E4" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("112X","An Unrestricted Line Officer who is qualified in Submarine Warfare","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('112X','An Unrestricted Line Officer who is qualified in Submarine Warfare','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7062,7 +7072,7 @@
       </c>
       <c r="E5" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("113X","An Unrestricted Line Officer who is qualified in Special Warfare","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('113X','An Unrestricted Line Officer who is qualified in Special Warfare','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7082,7 +7092,7 @@
       </c>
       <c r="E6" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("114X","An Unrestricted Line Officer who is qualified in Explosive Ordnance Disposal (EOD) Warfare","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('114X','An Unrestricted Line Officer who is qualified in Explosive Ordnance Disposal (EOD) Warfare','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7102,7 +7112,7 @@
       </c>
       <c r="E7" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("116X","Unrestricted Line Officer who is in training for Surface Warfare qualification","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('116X','Unrestricted Line Officer who is in training for Surface Warfare qualification','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7122,7 +7132,7 @@
       </c>
       <c r="E8" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("117X","Unrestricted Line Officer who is in training for Submarine Warfare qualification","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('117X','Unrestricted Line Officer who is in training for Submarine Warfare qualification','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7142,7 +7152,7 @@
       </c>
       <c r="E9" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("118X","Unrestricted Line Officer who is in training for Special Warfare qualification","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('118X','Unrestricted Line Officer who is in training for Special Warfare qualification','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7162,10 +7172,10 @@
       </c>
       <c r="E10" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("119X","Unrestricted Line Officer who is in training for Explosive Ordnance Disposal qualification","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="84" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('119X','Unrestricted Line Officer who is in training for Explosive Ordnance Disposal qualification','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="70" x14ac:dyDescent="0.2">
       <c r="A11" s="21" t="s">
         <v>46</v>
       </c>
@@ -7182,7 +7192,7 @@
       </c>
       <c r="E11" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("120X","Special Duty Officer - Human Resource Officer A Restricted Line Officer of the Human Resources Community who will plan, program and execute life-cycle management of our Navy's most important resource - people.","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('120X','Special Duty Officer - Human Resource Officer A Restricted Line Officer of the Human Resources Community who will plan, program and execute life-cycle management of our Navy''s most important resource - people.','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7202,7 +7212,7 @@
       </c>
       <c r="E12" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("121X","Restricted Line Officer (Nuclear Power School Instructor) regulated by Program Authorization 100B.","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('121X','Restricted Line Officer (Nuclear Power School Instructor) regulated by Program Authorization 100B.','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7222,7 +7232,7 @@
       </c>
       <c r="E13" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("1230","Restricted Line Officer (Permanent Military Professor) regulated by OPNAVINST 1520.40","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('1230','Restricted Line Officer (Permanent Military Professor) regulated by OPNAVINST 1520.40','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7242,10 +7252,10 @@
       </c>
       <c r="E14" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("128X","Special Duty Officer-Permanent Professional Recruiter Officer (Reserve Recruiting) (LT and LCDR)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="98" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('128X','Special Duty Officer-Permanent Professional Recruiter Officer (Reserve Recruiting) (LT and LCDR)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="70" x14ac:dyDescent="0.2">
       <c r="A15" s="21" t="s">
         <v>61</v>
       </c>
@@ -7262,10 +7272,10 @@
       </c>
       <c r="E15" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("130X","An Unrestricted Line Officer who is a member of the aeronautical community and whose rating as a pilot or NFO has been terminated. (These officers may be assigned to 1000, 1050, 1300, 1310 or 1320 designated billets, if otherwise qualified.)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="70" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('130X','An Unrestricted Line Officer who is a member of the aeronautical community and whose rating as a pilot or NFO has been terminated. (These officers may be assigned to 1000, 1050, 1300, 1310 or 1320 designated billets, if otherwise qualified.)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A16" s="21" t="s">
         <v>69</v>
       </c>
@@ -7282,10 +7292,10 @@
       </c>
       <c r="E16" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("131X","An Unrestricted Line Officer who is qualified for duty involving flying heavier-than-air, or heavier and lighter-than-air type of aircraft as a pilot","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="70" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('131X','An Unrestricted Line Officer who is qualified for duty involving flying heavier-than-air, or heavier and lighter-than-air type of aircraft as a pilot','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A17" s="21" t="s">
         <v>78</v>
       </c>
@@ -7302,7 +7312,7 @@
       </c>
       <c r="E17" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("132X","An Unrestricted Line Officer who is qualified for duty involving flying heavier-than-air or heavier and lighter-than-air type aircraft as a Naval Flight Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('132X','An Unrestricted Line Officer who is qualified for duty involving flying heavier-than-air or heavier and lighter-than-air type aircraft as a Naval Flight Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7322,7 +7332,7 @@
       </c>
       <c r="E18" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("137X","An Unrestricted Line Officer who is in training for duty involving flying as a Naval Flight Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('137X','An Unrestricted Line Officer who is in training for duty involving flying as a Naval Flight Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7342,10 +7352,10 @@
       </c>
       <c r="E19" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("139X","An Unrestricted Line Officer who is in training for duty involving flying as a pilot","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="98" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('139X','An Unrestricted Line Officer who is in training for duty involving flying as a pilot','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="84" x14ac:dyDescent="0.2">
       <c r="A20" s="21" t="s">
         <v>96</v>
       </c>
@@ -7362,7 +7372,7 @@
       </c>
       <c r="E20" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("144X","Engineering Duty Officer who is qualified as a Ship Engineering specialist IAW MILPERSMAN 1210-190. They include specialists in Ship and Ship systems Engineering, Electronic Systems Engineering, Combat/Weapons Systems Engineering, and Ordnance Systems Engineering","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('144X','Engineering Duty Officer who is qualified as a Ship Engineering specialist IAW MILPERSMAN 1210-190. They include specialists in Ship and Ship systems Engineering, Electronic Systems Engineering, Combat/Weapons Systems Engineering, and Ordnance Systems Engineering','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7382,10 +7392,10 @@
       </c>
       <c r="E21" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("146X","Engineering Duty Officer who is in the process of completing the prescribed program leading to designation as 144X","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="84" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('146X','Engineering Duty Officer who is in the process of completing the prescribed program leading to designation as 144X','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A22" s="21" t="s">
         <v>106</v>
       </c>
@@ -7402,7 +7412,7 @@
       </c>
       <c r="E22" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("150X","A Restricted Line AED Flag Officer or Captain who was formerly either an AED officer (Aerospace Engineering--designator 151X) or an AMD officer (Aviation Maintenance--designator 152X)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('150X','A Restricted Line AED Flag Officer or Captain who was formerly either an AED officer (Aerospace Engineering--designator 151X) or an AMD officer (Aviation Maintenance--designator 152X)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7422,10 +7432,10 @@
       </c>
       <c r="E23" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("151X","Aerospace Engineering Duty Officer (Aerospace Engineering)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('151X','Aerospace Engineering Duty Officer (Aerospace Engineering)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A24" s="21" t="s">
         <v>115</v>
       </c>
@@ -7442,10 +7452,10 @@
       </c>
       <c r="E24" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("154X","Aviation Duty Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('154X','Aviation Duty Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A25" s="21" t="s">
         <v>127</v>
       </c>
@@ -7462,7 +7472,7 @@
       </c>
       <c r="E25" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("165X","Special Duty Officer - Public Affairs","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('165X','Special Duty Officer - Public Affairs','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7482,10 +7492,10 @@
       </c>
       <c r="E26" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("166X","Special Duty Officer – Strategic Sealift Officer (SSO)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('166X','Special Duty Officer – Strategic Sealift Officer (SSO)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A27" s="21" t="s">
         <v>134</v>
       </c>
@@ -7502,7 +7512,7 @@
       </c>
       <c r="E27" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("168X","Special Duty Officer (Reserve Recruiting)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('168X','Special Duty Officer (Reserve Recruiting)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7522,10 +7532,10 @@
       </c>
       <c r="E28" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("171X","Special Duty Officer qualified as a Foreign Area Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('171X','Special Duty Officer qualified as a Foreign Area Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A29" s="21" t="s">
         <v>144</v>
       </c>
@@ -7542,7 +7552,7 @@
       </c>
       <c r="E29" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("180X","Information Warfare Line Officer - Oceanography","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('180X','Information Warfare Line Officer - Oceanography','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7562,7 +7572,7 @@
       </c>
       <c r="E30" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("181X","Information Warfare Line Officer – Cryptologic Warfare Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('181X','Information Warfare Line Officer – Cryptologic Warfare Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7582,7 +7592,7 @@
       </c>
       <c r="E31" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("182X","Information Warfare Line Officer – Information Professional Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('182X','Information Warfare Line Officer – Information Professional Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7602,7 +7612,7 @@
       </c>
       <c r="E32" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("183X","Information Warfare Line Officer– Intelligence Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('183X','Information Warfare Line Officer– Intelligence Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7622,10 +7632,10 @@
       </c>
       <c r="E33" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("184X","Information Warfare Line Officer– Cyber Warfare Engineer","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('184X','Information Warfare Line Officer– Cyber Warfare Engineer','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A34" s="21" t="s">
         <v>152</v>
       </c>
@@ -7642,7 +7652,7 @@
       </c>
       <c r="E34" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("186X","Information Warfare Line Officer – IWC Flag Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('186X','Information Warfare Line Officer – IWC Flag Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7662,7 +7672,7 @@
       </c>
       <c r="E35" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("187X","Information Warfare Line Officer - Maritime Space Officer / Reserve Grades URL/RL O2 to O6","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('187X','Information Warfare Line Officer - Maritime Space Officer / Reserve Grades URL/RL O2 to O6','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7682,7 +7692,7 @@
       </c>
       <c r="E36" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("188X","Information Warfare Line Officer -Maritime Cyber Warfare Officer (O1 to O6)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('188X','Information Warfare Line Officer -Maritime Cyber Warfare Officer (O1 to O6)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7702,7 +7712,7 @@
       </c>
       <c r="E37" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("190X","An Unrestricted Line Officer under instruction as a prospective Nurse Corps officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('190X','An Unrestricted Line Officer under instruction as a prospective Nurse Corps officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7722,7 +7732,7 @@
       </c>
       <c r="E38" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("191X","An Unrestricted Line Officer under instruction as a prospective Medical Corps officer (Senior Medical Student)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('191X','An Unrestricted Line Officer under instruction as a prospective Medical Corps officer (Senior Medical Student)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7742,7 +7752,7 @@
       </c>
       <c r="E39" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("192X","An Unrestricted Line Officer under instruction as a prospective Dental Corps officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('192X','An Unrestricted Line Officer under instruction as a prospective Dental Corps officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7762,7 +7772,7 @@
       </c>
       <c r="E40" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("193X","An Unrestricted Line Officer under instruction as a prospective Medical Service officer (Optometry)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('193X','An Unrestricted Line Officer under instruction as a prospective Medical Service officer (Optometry)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7782,7 +7792,7 @@
       </c>
       <c r="E41" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("194X","An Unrestricted Line Officer under instruction as a prospective Chaplain Corps officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('194X','An Unrestricted Line Officer under instruction as a prospective Chaplain Corps officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7802,10 +7812,10 @@
       </c>
       <c r="E42" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("195X","An Unrestricted Line Officer under instruction as a prospective Judge Advocate General's Corps officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" ht="70" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('195X','An Unrestricted Line Officer under instruction as a prospective Judge Advocate General''s Corps officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A43" s="21" t="s">
         <v>176</v>
       </c>
@@ -7822,10 +7832,10 @@
       </c>
       <c r="E43" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("196X","An Unrestricted Line Officer under instruction as a prospective Medical Corps officer (Medical /Osteopathic Scholarship Program)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" ht="70" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('196X','An Unrestricted Line Officer under instruction as a prospective Medical Corps officer (Medical /Osteopathic Scholarship Program)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A44" s="21" t="s">
         <v>178</v>
       </c>
@@ -7842,10 +7852,10 @@
       </c>
       <c r="E44" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("197X","An Unrestricted Line Officer under instruction in the Armed Forces Health Professions Scholarship Program (Medical/Osteopathic)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" ht="70" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('197X','An Unrestricted Line Officer under instruction in the Armed Forces Health Professions Scholarship Program (Medical/Osteopathic)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A45" s="21" t="s">
         <v>180</v>
       </c>
@@ -7862,10 +7872,10 @@
       </c>
       <c r="E45" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("198X","An Unrestricted Line Officer under instruction in the Armed Forces Health Professions Scholarship Program (Dental)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" ht="70" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('198X','An Unrestricted Line Officer under instruction in the Armed Forces Health Professions Scholarship Program (Dental)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A46" s="21" t="s">
         <v>182</v>
       </c>
@@ -7882,10 +7892,10 @@
       </c>
       <c r="E46" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("199X","An Unrestricted Line Officer under instruction in the Armed Forces Health Professions Scholarship Program (Medical Service Corps)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('199X','An Unrestricted Line Officer under instruction in the Armed Forces Health Professions Scholarship Program (Medical Service Corps)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A47" s="21" t="s">
         <v>190</v>
       </c>
@@ -7902,10 +7912,10 @@
       </c>
       <c r="E47" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("210X","A Medical Corps Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('210X','A Medical Corps Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A48" s="21" t="s">
         <v>195</v>
       </c>
@@ -7922,10 +7932,10 @@
       </c>
       <c r="E48" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("220X","A Dental Corps Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('220X','A Dental Corps Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A49" s="21" t="s">
         <v>198</v>
       </c>
@@ -7942,10 +7952,10 @@
       </c>
       <c r="E49" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("230X","A Medical Service Corps Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('230X','A Medical Service Corps Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A50" s="21" t="s">
         <v>203</v>
       </c>
@@ -7962,7 +7972,7 @@
       </c>
       <c r="E50" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("250X","A Judge Advocate General Corps Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('250X','A Judge Advocate General Corps Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -7982,10 +7992,10 @@
       </c>
       <c r="E51" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("270X","Active duty Nurse Corps, Medical Service Corps, Medical Corps, and Dental Corps officer in rank of O7","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('270X','Active duty Nurse Corps, Medical Service Corps, Medical Corps, and Dental Corps officer in rank of O7','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A52" s="21" t="s">
         <v>208</v>
       </c>
@@ -8002,10 +8012,10 @@
       </c>
       <c r="E52" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("290X","A Nurse Corps Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('290X','A Nurse Corps Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A53" s="21" t="s">
         <v>211</v>
       </c>
@@ -8022,7 +8032,7 @@
       </c>
       <c r="E53" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("310X","A Supply Corps Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('310X','A Supply Corps Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -8042,10 +8052,10 @@
       </c>
       <c r="E54" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("316X","A direct commissioned Supply Corps Officer in training for qualification","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('316X','A direct commissioned Supply Corps Officer in training for qualification','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A55" s="21" t="s">
         <v>217</v>
       </c>
@@ -8062,10 +8072,10 @@
       </c>
       <c r="E55" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("410X","A Chaplain Corps Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('410X','A Chaplain Corps Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A56" s="21" t="s">
         <v>220</v>
       </c>
@@ -8082,10 +8092,10 @@
       </c>
       <c r="E56" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("510X","A Civil Engineer Corps Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('510X','A Civil Engineer Corps Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A57" s="21" t="s">
         <v>226</v>
       </c>
@@ -8102,10 +8112,10 @@
       </c>
       <c r="E57" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("611X","A Limited Duty Officer (Deck - Surface)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('611X','A Limited Duty Officer (Deck - Surface)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A58" s="21" t="s">
         <v>229</v>
       </c>
@@ -8122,7 +8132,7 @@
       </c>
       <c r="E58" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("612X","A Limited Duty Officer (Operations - Surface)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('612X','A Limited Duty Officer (Operations - Surface)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -8142,10 +8152,10 @@
       </c>
       <c r="E59" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("613X","A Limited Duty Officer (Engineering/Repair - Surface)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('613X','A Limited Duty Officer (Engineering/Repair - Surface)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A60" s="21" t="s">
         <v>235</v>
       </c>
@@ -8162,7 +8172,7 @@
       </c>
       <c r="E60" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("618X","A Limited Duty Officer (Electronics - Surface)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('618X','A Limited Duty Officer (Electronics - Surface)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -8182,7 +8192,7 @@
       </c>
       <c r="E61" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("620X","A Limited Duty Officer (Nuclear Power); Formerly DESIG 640X","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('620X','A Limited Duty Officer (Nuclear Power); Formerly DESIG 640X','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -8202,10 +8212,10 @@
       </c>
       <c r="E62" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("623X","A Limited Duty Officer (Engineering/Repair - Submarine)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('623X','A Limited Duty Officer (Engineering/Repair - Submarine)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A63" s="21" t="s">
         <v>244</v>
       </c>
@@ -8222,10 +8232,10 @@
       </c>
       <c r="E63" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("626X","A Limited Duty Officer (Ordnance - Submarine)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('626X','A Limited Duty Officer (Ordnance - Submarine)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A64" s="21" t="s">
         <v>247</v>
       </c>
@@ -8242,7 +8252,7 @@
       </c>
       <c r="E64" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("628X","A Limited Duty Officer (Electronics - Submarine)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('628X','A Limited Duty Officer (Electronics - Submarine)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -8262,10 +8272,10 @@
       </c>
       <c r="E65" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("629X","A Limited Duty Officer (Communications - Submarine)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('629X','A Limited Duty Officer (Communications - Submarine)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A66" s="21" t="s">
         <v>256</v>
       </c>
@@ -8282,10 +8292,10 @@
       </c>
       <c r="E66" s="21" t="str">
         <f t="shared" si="2"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("631X","A Limited Duty Officer (Aviation Deck)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('631X','A Limited Duty Officer (Aviation Deck)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A67" s="21" t="s">
         <v>259</v>
       </c>
@@ -8301,11 +8311,13 @@
         <v xml:space="preserve">						{"632X", "A Limited Duty Officer (Aviation Operations)"},</v>
       </c>
       <c r="E67" s="21" t="str">
-        <f t="shared" ref="E67:E105" si="6">+_xlfn.CONCAT("insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values (""",B67,""",""",TRIM(C67),""",""NAVPERS 15839I VOL I (JAN 2026)"");")</f>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("632X","A Limited Duty Officer (Aviation Operations)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <f t="shared" ref="E67:E105" si="6">"insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('"
+ &amp; SUBSTITUTE(B67, "'", "''") &amp; "','"
+ &amp; SUBSTITUTE(TRIM(C67), "'", "''") &amp; "','NAVPERS 15839I VOL I (JAN 2026)');"</f>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('632X','A Limited Duty Officer (Aviation Operations)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A68" s="21" t="s">
         <v>264</v>
       </c>
@@ -8322,10 +8334,10 @@
       </c>
       <c r="E68" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("633X","A Limited Duty Officer (Aviation Maintenance)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('633X','A Limited Duty Officer (Aviation Maintenance)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A69" s="21" t="s">
         <v>267</v>
       </c>
@@ -8342,10 +8354,10 @@
       </c>
       <c r="E69" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("636X","A Limited Duty Officer (Aviation Ordnance)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('636X','A Limited Duty Officer (Aviation Ordnance)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A70" s="21" t="s">
         <v>270</v>
       </c>
@@ -8362,10 +8374,10 @@
       </c>
       <c r="E70" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("639X","A Limited Duty Officer (Air Traffic Control)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('639X','A Limited Duty Officer (Air Traffic Control)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A71" s="21" t="s">
         <v>274</v>
       </c>
@@ -8382,10 +8394,10 @@
       </c>
       <c r="E71" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("641X","A Limited Duty Officer (Administration)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('641X','A Limited Duty Officer (Administration)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A72" s="21" t="s">
         <v>277</v>
       </c>
@@ -8402,7 +8414,7 @@
       </c>
       <c r="E72" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("643X","A Limited Duty Officer (Bandmaster)","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('643X','A Limited Duty Officer (Bandmaster)','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -8422,10 +8434,10 @@
       </c>
       <c r="E73" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("648X","A Limited Duty Officer (Explosive Ordnance Disposal)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('648X','A Limited Duty Officer (Explosive Ordnance Disposal)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A74" s="21" t="s">
         <v>283</v>
       </c>
@@ -8442,10 +8454,10 @@
       </c>
       <c r="E74" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("649X","A Limited Duty Officer (Security)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('649X','A Limited Duty Officer (Security)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A75" s="21" t="s">
         <v>291</v>
       </c>
@@ -8462,10 +8474,10 @@
       </c>
       <c r="E75" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("651X","A Limited Duty Officer of the Supply Corps","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('651X','A Limited Duty Officer of the Supply Corps','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A76" s="21" t="s">
         <v>294</v>
       </c>
@@ -8482,7 +8494,7 @@
       </c>
       <c r="E76" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("653X","A Limited Duty Officer of the Civil Engineer Corps","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('653X','A Limited Duty Officer of the Civil Engineer Corps','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -8502,7 +8514,7 @@
       </c>
       <c r="E77" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("680X","A Limited Duty Officer (Meteorology/Oceanography) Formerly DESIG 646X","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('680X','A Limited Duty Officer (Meteorology/Oceanography) Formerly DESIG 646X','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -8522,7 +8534,7 @@
       </c>
       <c r="E78" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("681X","A Limited Duty Officer (Cryptologic Warfare) Formerly DESIG 644X","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('681X','A Limited Duty Officer (Cryptologic Warfare) Formerly DESIG 644X','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -8542,7 +8554,7 @@
       </c>
       <c r="E79" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("682X","A Limited Duty Officer (Information Professional) Formerly DESIG 642X","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('682X','A Limited Duty Officer (Information Professional) Formerly DESIG 642X','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -8562,10 +8574,10 @@
       </c>
       <c r="E80" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("683X","A Limited Duty Officer (Intelligence) Formerly DESIG 645X","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('683X','A Limited Duty Officer (Intelligence) Formerly DESIG 645X','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A81" s="21" t="s">
         <v>312</v>
       </c>
@@ -8582,10 +8594,10 @@
       </c>
       <c r="E81" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("711X","Boatswain (Surface)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('711X','Boatswain (Surface)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A82" s="21" t="s">
         <v>315</v>
       </c>
@@ -8602,10 +8614,10 @@
       </c>
       <c r="E82" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("712X","Operations Technician (Surface)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('712X','Operations Technician (Surface)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A83" s="21" t="s">
         <v>318</v>
       </c>
@@ -8622,10 +8634,10 @@
       </c>
       <c r="E83" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("713X","Engineering Technician (Surface)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('713X','Engineering Technician (Surface)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A84" s="21" t="s">
         <v>321</v>
       </c>
@@ -8642,10 +8654,10 @@
       </c>
       <c r="E84" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("715X","Special Warfare Technician","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" ht="70" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('715X','Special Warfare Technician','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A85" s="21" t="s">
         <v>324</v>
       </c>
@@ -8662,10 +8674,10 @@
       </c>
       <c r="E85" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("717X","A Chief Warrant Officer with sophisticated, technical knowledge in all aspects of the Naval Special Warfare Combat Crewman","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('717X','A Chief Warrant Officer with sophisticated, technical knowledge in all aspects of the Naval Special Warfare Combat Crewman','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A86" s="21" t="s">
         <v>327</v>
       </c>
@@ -8682,10 +8694,10 @@
       </c>
       <c r="E86" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("718X","Electronics Technician (Surface)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('718X','Electronics Technician (Surface)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A87" s="21" t="s">
         <v>331</v>
       </c>
@@ -8702,10 +8714,10 @@
       </c>
       <c r="E87" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("720X","Diving Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('720X','Diving Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A88" s="21" t="s">
         <v>334</v>
       </c>
@@ -8722,10 +8734,10 @@
       </c>
       <c r="E88" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("726X","Ordnance Technician (Submarine)","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('726X','Ordnance Technician (Submarine)','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A89" s="21" t="s">
         <v>337</v>
       </c>
@@ -8742,10 +8754,10 @@
       </c>
       <c r="E89" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("728X","Acoustic Technician","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('728X','Acoustic Technician','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A90" s="21" t="s">
         <v>341</v>
       </c>
@@ -8762,10 +8774,10 @@
       </c>
       <c r="E90" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("731X","Aviation Boatswain","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('731X','Aviation Boatswain','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A91" s="21" t="s">
         <v>344</v>
       </c>
@@ -8782,10 +8794,10 @@
       </c>
       <c r="E91" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("732X","Aviation Operations Technician","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('732X','Aviation Operations Technician','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A92" s="21" t="s">
         <v>349</v>
       </c>
@@ -8802,10 +8814,10 @@
       </c>
       <c r="E92" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("733X","Aviation Maintenance Technician","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('733X','Aviation Maintenance Technician','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A93" s="21" t="s">
         <v>352</v>
       </c>
@@ -8822,10 +8834,10 @@
       </c>
       <c r="E93" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("736X","Aviation Ordnance Technician","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('736X','Aviation Ordnance Technician','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A94" s="21" t="s">
         <v>355</v>
       </c>
@@ -8842,10 +8854,10 @@
       </c>
       <c r="E94" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("737X","Air Vehicle Pilot","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('737X','Air Vehicle Pilot','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A95" s="21" t="s">
         <v>358</v>
       </c>
@@ -8862,10 +8874,10 @@
       </c>
       <c r="E95" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("740X","Nuclear Power Technician","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('740X','Nuclear Power Technician','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A96" s="21" t="s">
         <v>361</v>
       </c>
@@ -8882,10 +8894,10 @@
       </c>
       <c r="E96" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("741X","Ship's Clerk","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('741X','Ship''s Clerk','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A97" s="21" t="s">
         <v>364</v>
       </c>
@@ -8902,10 +8914,10 @@
       </c>
       <c r="E97" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("749X","Security Technician","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('749X','Security Technician','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A98" s="21" t="s">
         <v>371</v>
       </c>
@@ -8922,10 +8934,10 @@
       </c>
       <c r="E98" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("752X","Food Service Warrant","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('752X','Food Service Warrant','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A99" s="21" t="s">
         <v>374</v>
       </c>
@@ -8942,10 +8954,10 @@
       </c>
       <c r="E99" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("753X","Civil Engineering Warrant","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('753X','Civil Engineering Warrant','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A100" s="21" t="s">
         <v>377</v>
       </c>
@@ -8962,10 +8974,10 @@
       </c>
       <c r="E100" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("756X","Technical Nurse","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('756X','Technical Nurse','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A101" s="21" t="s">
         <v>383</v>
       </c>
@@ -8982,7 +8994,7 @@
       </c>
       <c r="E101" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("780X","Oceanography Warrant Officer","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('780X','Oceanography Warrant Officer','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="102" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -9002,7 +9014,7 @@
       </c>
       <c r="E102" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("781X","Cryptologic Warfare Technician Formerly DESIG 744X","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('781X','Cryptologic Warfare Technician Formerly DESIG 744X','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="103" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -9022,10 +9034,10 @@
       </c>
       <c r="E103" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("782X","Information Systems Technician Formerly DESIG 742X","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('782X','Information Systems Technician Formerly DESIG 742X','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A104" s="21" t="s">
         <v>390</v>
       </c>
@@ -9042,10 +9054,10 @@
       </c>
       <c r="E104" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("783X","Intelligence Technician Formerly DESIG 745X","NAVPERS 15839I VOL I (JAN 2026)");</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('783X','Intelligence Technician Formerly DESIG 745X','NAVPERS 15839I VOL I (JAN 2026)');</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A105" s="21" t="s">
         <v>392</v>
       </c>
@@ -9062,7 +9074,7 @@
       </c>
       <c r="E105" s="21" t="str">
         <f t="shared" si="6"/>
-        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ("784X","Cyber Warrant Officer Formerly DESIG 743X","NAVPERS 15839I VOL I (JAN 2026)");</v>
+        <v>insert into FTS_officer_designator_codes (suggest_text_1, suggest_text_2, source) values ('784X','Cyber Warrant Officer Formerly DESIG 743X','NAVPERS 15839I VOL I (JAN 2026)');</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
@@ -9436,6 +9448,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010040A4222558E32F46A7B24662BCB9CB1E" ma:contentTypeVersion="8" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="dca824fd6bc70765305ebc2bf07c9e8e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5dc2986f-9199-4b50-8f94-f34c80f8e7ca" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="04f40b43849b657032e89762f4b1b713" ns2:_="">
     <xsd:import namespace="5dc2986f-9199-4b50-8f94-f34c80f8e7ca"/>
@@ -9603,15 +9624,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -9619,6 +9631,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{36A6BBA7-6871-4353-9C6B-FBE0D066E1BE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{074DFEEE-09A0-4033-8313-F0DEEF422A97}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9632,14 +9652,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{36A6BBA7-6871-4353-9C6B-FBE0D066E1BE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>